<commit_message>
update 'inline block' of verigen doc.
</commit_message>
<xml_diff>
--- a/Common/doc/verigen/media/instruction_module.xlsx
+++ b/Common/doc/verigen/media/instruction_module.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\Profiles\Common\doc\verigen\media\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C84998DF-61D4-40B6-9866-469A162A8082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A902DABF-3076-4D1F-9D0B-A3EDD9B262CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4380" yWindow="2175" windowWidth="21465" windowHeight="13425" firstSheet="10" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" firstSheet="10" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="6" r:id="rId1"/>
@@ -56,6 +56,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -569,10 +572,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Module source to be a sub module</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Sub module name.
 If omitted, it is named the same as the original module name.
 If there are several omitted sub modules with the same name, put a number in the form of "_#" after each name to avoid duplication.</t>
@@ -668,6 +667,10 @@
   <si>
     <t>The modport name, if used for internal declarations other than ports.
 Do not specify this value. And if 'I' is modport, then this 'modport must be nil.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Module source to be a sub module or name</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1004,13 +1007,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63D1552F-D2B8-4AD9-9ECE-3CAF9162E459}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.25" customWidth="1"/>
     <col min="3" max="3" width="33.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -1021,7 +1024,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1032,7 +1035,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1043,7 +1046,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -1054,7 +1057,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1065,7 +1068,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1076,7 +1079,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1087,7 +1090,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -1098,7 +1101,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -1109,7 +1112,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -1120,7 +1123,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A11" t="s">
         <v>63</v>
       </c>
@@ -1131,7 +1134,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1142,7 +1145,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1153,7 +1156,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1164,7 +1167,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1175,7 +1178,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A16" t="s">
         <v>55</v>
       </c>
@@ -1186,18 +1189,18 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A18" t="s">
         <v>10</v>
       </c>
@@ -1208,7 +1211,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -1219,7 +1222,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A20" t="s">
         <v>59</v>
       </c>
@@ -1230,7 +1233,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -1251,13 +1254,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A75E32B-39FA-48AF-B4E1-579B635CE77E}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1265,15 +1268,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1281,28 +1284,28 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B5" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="66" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1315,13 +1318,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4872EA8D-C206-4975-8F57-5608D1E780D6}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1329,7 +1332,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -1337,7 +1340,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1345,7 +1348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -1353,7 +1356,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>36</v>
       </c>
@@ -1371,13 +1374,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B50024F-C566-4A8D-B5DE-B9604581D8DC}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1385,7 +1388,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -1393,7 +1396,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1401,7 +1404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="50.65" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -1409,7 +1412,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1427,13 +1430,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{928081EA-571E-4518-9D8A-1567A1472513}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1441,7 +1444,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -1449,7 +1452,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1457,7 +1460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -1465,7 +1468,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1473,7 +1476,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>39</v>
       </c>
@@ -1481,7 +1484,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>40</v>
       </c>
@@ -1499,13 +1502,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD855936-E57A-4AAE-A547-E3F2DF4F0374}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1513,7 +1516,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -1521,7 +1524,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1529,7 +1532,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -1537,7 +1540,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1555,13 +1558,13 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3D7D268-AD21-44BB-8182-E394A1BAB6BC}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1569,7 +1572,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -1577,7 +1580,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1585,7 +1588,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -1593,15 +1596,15 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="33" x14ac:dyDescent="0.3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1609,12 +1612,12 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="66" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="67.5" x14ac:dyDescent="0.6">
       <c r="A7" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -1627,13 +1630,13 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3BA6C9D-83F7-41AC-A15F-DD0842A0B82E}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1641,7 +1644,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -1649,7 +1652,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1657,7 +1660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -1665,7 +1668,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>65</v>
       </c>
@@ -1682,13 +1685,13 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5785E4B8-2D74-44E5-B491-19BF525ABA02}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1696,7 +1699,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -1704,7 +1707,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1712,7 +1715,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="33" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -1720,7 +1723,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1738,13 +1741,13 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA580444-854B-4B19-9F3C-A3C0598A14F6}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1752,7 +1755,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -1760,7 +1763,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1768,7 +1771,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="33" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="33.75" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -1776,7 +1779,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1794,13 +1797,13 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E82B7A0-A94F-47BE-ACEE-BBB2DA8903FA}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1808,7 +1811,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -1816,7 +1819,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1824,7 +1827,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -1832,20 +1835,20 @@
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="82.5" x14ac:dyDescent="0.3">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="84.4" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1858,13 +1861,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12A76216-2298-479D-87E6-5C639887A995}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.25" customWidth="1"/>
     <col min="3" max="3" width="33.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -1875,7 +1878,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1886,7 +1889,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1897,7 +1900,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1908,7 +1911,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -1919,7 +1922,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -1930,7 +1933,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.6">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1950,13 +1953,13 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01B9B674-2006-4921-91E8-F776B72473CB}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1964,7 +1967,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -1972,7 +1975,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -1980,20 +1983,20 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2006,13 +2009,13 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28113802-B713-49E4-A818-7E4C797F3E8E}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2020,7 +2023,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2028,7 +2031,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2036,20 +2039,20 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="99" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="101.25" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -2061,13 +2064,13 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A772622C-72EA-4547-94FE-9EA66C7FB6BE}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2075,7 +2078,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2083,7 +2086,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2091,15 +2094,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -2107,12 +2110,12 @@
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -2125,13 +2128,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F508A2DE-DD70-49F7-944A-ED879E70751B}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2139,7 +2142,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2147,7 +2150,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2155,15 +2158,15 @@
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -2181,13 +2184,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1F942EC-D9CE-4518-8AE9-9DD2A68C7F6E}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2195,7 +2198,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2203,7 +2206,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2211,28 +2214,28 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2245,13 +2248,13 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3433696-309F-48A2-94BE-A5A058FB822B}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2259,7 +2262,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2267,28 +2270,28 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -2301,13 +2304,13 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F1D0C89-3871-4B99-A935-D12B0A533798}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2315,7 +2318,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2323,7 +2326,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2331,20 +2334,20 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -2356,13 +2359,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2370,7 +2373,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2378,7 +2381,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2386,7 +2389,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -2394,7 +2397,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -2412,13 +2415,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1E26BB1-25FB-4478-A7EA-E4CE5AFF0184}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2426,7 +2429,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2434,7 +2437,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2442,7 +2445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="118.15" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -2460,13 +2463,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74775AB0-90E6-4F96-93BF-E413632C7F79}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2474,7 +2477,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2482,7 +2485,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2490,7 +2493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="132" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -2498,7 +2501,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>32</v>
       </c>
@@ -2515,13 +2518,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BDBF1A7-2EF9-4A6E-97F7-6E6DC3263962}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2529,7 +2532,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2537,7 +2540,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2545,7 +2548,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -2553,7 +2556,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -2570,13 +2573,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB28CFE9-CB71-4320-83F8-E42AFA068774}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2584,7 +2587,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2592,7 +2595,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2600,7 +2603,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -2608,7 +2611,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2625,13 +2628,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4066CFF-428B-4723-A23B-AA045754B767}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2639,7 +2642,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2647,7 +2650,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2655,7 +2658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="165" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="168.75" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
@@ -2663,7 +2666,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A5" s="1" t="s">
         <v>32</v>
       </c>
@@ -2671,7 +2674,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -2689,13 +2692,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D19B922-7931-4B59-9944-8B3AC4588909}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="10.125" customWidth="1"/>
     <col min="2" max="2" width="55.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2703,7 +2706,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2711,7 +2714,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
@@ -2719,7 +2722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.6">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>

</xml_diff>